<commit_message>
Fix 1991 batting headers: K% was mislabeled as SB
Original transcription dropped the K% column header but left the K%
values in place, which shifted the SB/SAC/TB/E column labels by one
position. Result: every per-player SB read by the master extractor
was actually a K% (so Cherbas SB=19, Wark SB=33 in 3 AB, etc.).

Relabeled the Team Batting header so columns now read correctly:
  Player AB R H RBI 2B 3B HR BB HBP K K% SB SAC TB OBP AVG GP

E (errors) was never carried into the xlsx in the first place — the
original transcription dropped it entirely. The new layout reflects
that.

Cross-checked against typed Individual Records for 1991:
  Cherbas/Dupuis SB=6 ✓, Peschek TB=36 ✓, Hoskins BB=10 ✓, all
  other top-line records intact.

1990 verified separately — its source has no K% column and existing
data matches the typed records (no fix needed).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Historical/1991/1991_Season_Stats.xlsx
+++ b/Historical/1991/1991_Season_Stats.xlsx
@@ -979,7 +979,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Note: Some TB column values in the source don't sum cleanly to the visible 1B/2B/3B/HR breakdown — preserved as printed. Some narrow columns (HBP, SB, SAC, GP) had reading challenges for a few players; values are best-effort.</t>
+          <t>Note: Original 1991 source has 18 stat columns including K% between K and SB. Earlier transcription dropped the K% header label but left the K% values, which shifted SB/SAC/TB/E by one position. Header relabeled (2026-04-27) so the actual SB column reads correctly; E (errors) is no longer carried — its values were never preserved by the original transcription. Some TB column values still don't sum cleanly to the visible 1B/2B/3B/HR breakdown — preserved as printed. Some narrow columns (HBP, SB, SAC, GP) had reading challenges for a few players; values are best-effort.</t>
         </is>
       </c>
     </row>
@@ -1041,22 +1041,22 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
+          <t>K%</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>SAC</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>TB</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">

</xml_diff>